<commit_message>
Auto commit: 2026-09-03 16:30
</commit_message>
<xml_diff>
--- a/data/lookup/lqas_lookup.xlsx
+++ b/data/lookup/lqas_lookup.xlsx
@@ -3817,7 +3817,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3945,7 +3945,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3977,7 +3977,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -5017,7 +5017,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>bOPV, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -5049,7 +5049,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>bOPV, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -6505,7 +6505,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -6537,7 +6537,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -11093,7 +11093,7 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
@@ -11125,7 +11125,7 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
@@ -11413,7 +11413,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
@@ -12997,7 +12997,7 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D397" t="inlineStr">
@@ -13029,7 +13029,7 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D398" t="inlineStr">
@@ -13821,7 +13821,7 @@
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
@@ -13853,7 +13853,7 @@
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
@@ -14925,7 +14925,7 @@
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>bOPV, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
@@ -14957,7 +14957,7 @@
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>bOPV, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
@@ -15021,7 +15021,7 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>nOPV2, nOPV2 &amp; bOPV</t>
+          <t>nOPV2 &amp; bOPV</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">

</xml_diff>